<commit_message>
DGFT new notification add
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/ALL_PDF/DGFT POLICY - Copy.xlsx
+++ b/backend/PDF_DOC/ALL_PDF/DGFT POLICY - Copy.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE36B395-A610-413E-AC97-2C5315136F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01CBD7E3-2B9B-4FD7-933E-C9557D93F856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PUBLIC NOTICE" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="887">
   <si>
     <t>DGFT - PUBLIC NOTICE</t>
   </si>
@@ -2684,6 +2684,15 @@
   </si>
   <si>
     <t>Allocation of 8606 MTRV of raw cane sugar to USA under TRQ scheme for US fiscal year 2026-regarding.</t>
+  </si>
+  <si>
+    <t>TRADE NOTICE- 06/2026-27</t>
+  </si>
+  <si>
+    <t>Electronic filing and Issuance of Preferential Certificate of Origin (CoO) under India-Oman Comprehensive Economic Partnership Agreement (India-Oman CEPA) with effect from June 01, 2026 - regarding.</t>
+  </si>
+  <si>
+    <t>PUBLIC NOTICE- 13/2026-27</t>
   </si>
 </sst>
 </file>
@@ -2722,7 +2731,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2759,6 +2768,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -2781,7 +2796,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2912,6 +2927,14 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3194,7 +3217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O383"/>
+  <dimension ref="A1:O384"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -3235,34 +3258,34 @@
       <c r="A5" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="54" t="s">
-        <v>882</v>
-      </c>
-      <c r="C5" s="55" t="s">
+      <c r="B5" s="58" t="s">
+        <v>886</v>
+      </c>
+      <c r="C5" s="59" t="s">
         <v>819</v>
       </c>
-      <c r="D5" s="57" t="s">
-        <v>883</v>
-      </c>
-      <c r="E5" s="56">
-        <v>46164</v>
+      <c r="D5" s="61" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="60">
+        <v>46171</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="34" t="s">
-        <v>863</v>
-      </c>
-      <c r="C6" s="35" t="s">
+      <c r="B6" s="54" t="s">
+        <v>882</v>
+      </c>
+      <c r="C6" s="55" t="s">
         <v>819</v>
       </c>
-      <c r="D6" s="36" t="s">
-        <v>864</v>
-      </c>
-      <c r="E6" s="49">
-        <v>46156</v>
+      <c r="D6" s="57" t="s">
+        <v>883</v>
+      </c>
+      <c r="E6" s="56">
+        <v>46164</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3270,16 +3293,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C7" s="35" t="s">
         <v>819</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>28</v>
+        <v>864</v>
       </c>
       <c r="E7" s="49">
-        <v>46153</v>
+        <v>46156</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3287,84 +3310,84 @@
         <v>4</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="C8" s="35" t="s">
         <v>819</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>867</v>
+        <v>28</v>
       </c>
       <c r="E8" s="49">
         <v>46153</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>5</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="C9" s="35" t="s">
         <v>819</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="E9" s="49">
-        <v>46150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>6</v>
       </c>
-      <c r="B10" s="50" t="s">
-        <v>870</v>
-      </c>
-      <c r="C10" s="51" t="s">
+      <c r="B10" s="34" t="s">
+        <v>868</v>
+      </c>
+      <c r="C10" s="35" t="s">
         <v>819</v>
       </c>
-      <c r="D10" s="52" t="s">
-        <v>871</v>
-      </c>
-      <c r="E10" s="53">
-        <v>46147</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="D10" s="36" t="s">
+        <v>869</v>
+      </c>
+      <c r="E10" s="49">
+        <v>46150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>7</v>
       </c>
-      <c r="B11" s="34" t="s">
-        <v>859</v>
-      </c>
-      <c r="C11" s="35" t="s">
+      <c r="B11" s="50" t="s">
+        <v>870</v>
+      </c>
+      <c r="C11" s="51" t="s">
         <v>819</v>
       </c>
-      <c r="D11" s="36" t="s">
-        <v>860</v>
-      </c>
-      <c r="E11" s="40">
-        <v>46146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="52" t="s">
+        <v>871</v>
+      </c>
+      <c r="E11" s="53">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>8</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="C12" s="35" t="s">
         <v>819</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="E12" s="40">
-        <v>46142</v>
+        <v>46146</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3372,33 +3395,33 @@
         <v>9</v>
       </c>
       <c r="B13" s="34" t="s">
-        <v>840</v>
-      </c>
-      <c r="C13" s="35">
-        <v>2026</v>
+        <v>861</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>819</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>841</v>
+        <v>862</v>
       </c>
       <c r="E13" s="40">
-        <v>46129</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>10</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>836</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>819</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>837</v>
-      </c>
-      <c r="E14" s="48">
-        <v>46122</v>
+      <c r="B14" s="34" t="s">
+        <v>840</v>
+      </c>
+      <c r="C14" s="35">
+        <v>2026</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>841</v>
+      </c>
+      <c r="E14" s="40">
+        <v>46129</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3406,50 +3429,50 @@
         <v>11</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="C15" s="26" t="s">
         <v>819</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="E15" s="48">
         <v>46122</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>12</v>
       </c>
-      <c r="B16" t="s">
-        <v>822</v>
-      </c>
-      <c r="C16" s="8" t="s">
+      <c r="B16" s="32" t="s">
+        <v>838</v>
+      </c>
+      <c r="C16" s="26" t="s">
         <v>819</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>821</v>
-      </c>
-      <c r="E16" s="38">
-        <v>46119</v>
+      <c r="D16" s="33" t="s">
+        <v>839</v>
+      </c>
+      <c r="E16" s="48">
+        <v>46122</v>
       </c>
     </row>
     <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>13</v>
       </c>
-      <c r="B17" s="21" t="s">
-        <v>811</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>812</v>
-      </c>
-      <c r="E17" s="41">
-        <v>46111</v>
+      <c r="B17" t="s">
+        <v>822</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>819</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="E17" s="38">
+        <v>46119</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3457,16 +3480,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>791</v>
-      </c>
-      <c r="C18" s="24">
-        <v>2025</v>
+        <v>811</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>8</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>792</v>
+        <v>812</v>
       </c>
       <c r="E18" s="41">
-        <v>46105</v>
+        <v>46111</v>
       </c>
     </row>
     <row r="19" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3474,16 +3497,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>786</v>
-      </c>
-      <c r="C19" s="24" t="s">
-        <v>4</v>
+        <v>791</v>
+      </c>
+      <c r="C19" s="24">
+        <v>2025</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>787</v>
+        <v>792</v>
       </c>
       <c r="E19" s="41">
-        <v>46101</v>
+        <v>46105</v>
       </c>
     </row>
     <row r="20" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3491,71 +3514,68 @@
         <v>16</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="C20" s="24" t="s">
         <v>4</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>778</v>
+        <v>787</v>
       </c>
       <c r="E20" s="41">
-        <v>46087</v>
+        <v>46101</v>
       </c>
     </row>
     <row r="21" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>17</v>
       </c>
-      <c r="B21" s="31" t="s">
-        <v>779</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="31" t="s">
+      <c r="B21" s="21" t="s">
+        <v>788</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>778</v>
       </c>
-      <c r="E21" s="45">
+      <c r="E21" s="41">
         <v>46087</v>
       </c>
-      <c r="F21" s="30"/>
-    </row>
-    <row r="22" spans="1:15" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>18</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>754</v>
-      </c>
-      <c r="C22" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>755</v>
-      </c>
-      <c r="E22" s="42" t="s">
-        <v>853</v>
-      </c>
+      <c r="B22" s="31" t="s">
+        <v>779</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="31" t="s">
+        <v>778</v>
+      </c>
+      <c r="E22" s="45">
+        <v>46087</v>
+      </c>
+      <c r="F22" s="30"/>
     </row>
     <row r="23" spans="1:15" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>19</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="E23" s="42" t="s">
         <v>853</v>
-      </c>
-      <c r="O23" s="21" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="21" customFormat="1" x14ac:dyDescent="0.25">
@@ -3563,33 +3583,36 @@
         <v>20</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C24" s="24" t="s">
         <v>4</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="E24" s="42" t="s">
         <v>853</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O24" s="21" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>21</v>
       </c>
-      <c r="B25" t="s">
-        <v>386</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>382</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E25" s="38">
-        <v>46328</v>
+      <c r="B25" s="21" t="s">
+        <v>759</v>
+      </c>
+      <c r="C25" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>760</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>853</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -3597,16 +3620,16 @@
         <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>4</v>
+        <v>382</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="E26" s="38">
-        <v>46144</v>
+        <v>46328</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -3614,16 +3637,16 @@
         <v>23</v>
       </c>
       <c r="B27" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D27" t="s">
-        <v>5</v>
+      <c r="D27" s="3" t="s">
+        <v>378</v>
       </c>
       <c r="E27" s="38">
-        <v>46045</v>
+        <v>46144</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -3631,16 +3654,16 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D28" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E28" s="38">
-        <v>46038</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3648,16 +3671,16 @@
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>390</v>
-      </c>
-      <c r="C29" s="8">
-        <v>2026</v>
+        <v>389</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D29" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E29" s="38">
-        <v>46031</v>
+        <v>46038</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3665,13 +3688,13 @@
         <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C30" s="8">
         <v>2026</v>
       </c>
       <c r="D30" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E30" s="38">
         <v>46031</v>
@@ -3682,16 +3705,16 @@
         <v>27</v>
       </c>
       <c r="B31" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C31" s="8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E31" s="38">
-        <v>46022</v>
+        <v>46031</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -3699,16 +3722,16 @@
         <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>393</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>4</v>
+        <v>392</v>
+      </c>
+      <c r="C32" s="8">
+        <v>2025</v>
       </c>
       <c r="D32" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E32" s="38">
-        <v>46010</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -3716,16 +3739,16 @@
         <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D33" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E33" s="38">
-        <v>46008</v>
+        <v>46010</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -3733,13 +3756,13 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E34" s="38">
         <v>46008</v>
@@ -3750,16 +3773,16 @@
         <v>31</v>
       </c>
       <c r="B35" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D35" t="s">
-        <v>374</v>
+        <v>19</v>
       </c>
       <c r="E35" s="38">
-        <v>46002</v>
+        <v>46008</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -3767,16 +3790,16 @@
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>397</v>
-      </c>
-      <c r="C36" s="8">
-        <v>2025</v>
+        <v>396</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D36" t="s">
-        <v>20</v>
+        <v>374</v>
       </c>
       <c r="E36" s="38">
-        <v>46001</v>
+        <v>46002</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -3784,13 +3807,13 @@
         <v>33</v>
       </c>
       <c r="B37" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C37" s="8">
         <v>2025</v>
       </c>
       <c r="D37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E37" s="38">
         <v>46001</v>
@@ -3801,16 +3824,16 @@
         <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>399</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>4</v>
+        <v>398</v>
+      </c>
+      <c r="C38" s="8">
+        <v>2025</v>
       </c>
       <c r="D38" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E38" s="38">
-        <v>45992</v>
+        <v>46001</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -3818,13 +3841,13 @@
         <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E39" s="38">
         <v>45992</v>
@@ -3835,16 +3858,16 @@
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>401</v>
-      </c>
-      <c r="C40" s="8">
-        <v>2025</v>
+        <v>400</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D40" t="s">
-        <v>373</v>
+        <v>24</v>
       </c>
       <c r="E40" s="38">
-        <v>45981</v>
+        <v>45992</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -3852,16 +3875,16 @@
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>402</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>4</v>
+        <v>401</v>
+      </c>
+      <c r="C41" s="8">
+        <v>2025</v>
       </c>
       <c r="D41" t="s">
-        <v>27</v>
+        <v>373</v>
       </c>
       <c r="E41" s="38">
-        <v>45959</v>
+        <v>45981</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -3869,16 +3892,16 @@
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>403</v>
-      </c>
-      <c r="C42" s="8">
-        <v>2025</v>
+        <v>402</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D42" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E42" s="38">
-        <v>45958</v>
+        <v>45959</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -3886,13 +3909,13 @@
         <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C43" s="8">
         <v>2025</v>
       </c>
       <c r="D43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E43" s="38">
         <v>45958</v>
@@ -3903,16 +3926,16 @@
         <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>405</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>8</v>
+        <v>404</v>
+      </c>
+      <c r="C44" s="8">
+        <v>2025</v>
       </c>
       <c r="D44" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E44" s="38">
-        <v>45953</v>
+        <v>45958</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -3920,16 +3943,16 @@
         <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E45" s="38">
-        <v>45952</v>
+        <v>45953</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -3937,16 +3960,16 @@
         <v>42</v>
       </c>
       <c r="B46" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D46" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E46" s="38">
-        <v>45945</v>
+        <v>45952</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -3954,16 +3977,16 @@
         <v>43</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>407</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D47" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E47" s="38">
-        <v>45940</v>
+        <v>45945</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -3971,13 +3994,13 @@
         <v>44</v>
       </c>
       <c r="B48" t="s">
-        <v>408</v>
+        <v>38</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D48" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E48" s="38">
         <v>45940</v>
@@ -3988,16 +4011,16 @@
         <v>45</v>
       </c>
       <c r="B49" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D49" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E49" s="38">
-        <v>45933</v>
+        <v>45940</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -4005,16 +4028,16 @@
         <v>46</v>
       </c>
       <c r="B50" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E50" s="38">
-        <v>45931</v>
+        <v>45933</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -4022,16 +4045,16 @@
         <v>47</v>
       </c>
       <c r="B51" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D51" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E51" s="38">
-        <v>45909</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -4039,16 +4062,16 @@
         <v>48</v>
       </c>
       <c r="B52" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D52" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E52" s="38">
-        <v>45903</v>
+        <v>45909</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -4056,16 +4079,16 @@
         <v>49</v>
       </c>
       <c r="B53" t="s">
-        <v>413</v>
-      </c>
-      <c r="C53" s="8">
-        <v>2025</v>
+        <v>412</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D53" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E53" s="38">
-        <v>45895</v>
+        <v>45903</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -4073,16 +4096,16 @@
         <v>50</v>
       </c>
       <c r="B54" t="s">
-        <v>414</v>
-      </c>
-      <c r="C54" s="8" t="s">
-        <v>4</v>
+        <v>413</v>
+      </c>
+      <c r="C54" s="8">
+        <v>2025</v>
       </c>
       <c r="D54" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E54" s="38">
-        <v>45891</v>
+        <v>45895</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -4090,16 +4113,16 @@
         <v>51</v>
       </c>
       <c r="B55" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D55" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E55" s="38">
-        <v>45870</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -4107,16 +4130,16 @@
         <v>52</v>
       </c>
       <c r="B56" t="s">
-        <v>416</v>
-      </c>
-      <c r="C56" s="8">
-        <v>2025</v>
+        <v>415</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E56" s="38">
-        <v>45868</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -4124,16 +4147,16 @@
         <v>53</v>
       </c>
       <c r="B57" t="s">
-        <v>417</v>
-      </c>
-      <c r="C57" s="8" t="s">
-        <v>4</v>
+        <v>416</v>
+      </c>
+      <c r="C57" s="8">
+        <v>2025</v>
       </c>
       <c r="D57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E57" s="38">
-        <v>45867</v>
+        <v>45868</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -4141,16 +4164,16 @@
         <v>54</v>
       </c>
       <c r="B58" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D58" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E58" s="38">
-        <v>45860</v>
+        <v>45867</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -4158,16 +4181,16 @@
         <v>55</v>
       </c>
       <c r="B59" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D59" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E59" s="38">
-        <v>45846</v>
+        <v>45860</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -4175,16 +4198,16 @@
         <v>56</v>
       </c>
       <c r="B60" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D60" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E60" s="38">
-        <v>45833</v>
+        <v>45846</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -4192,13 +4215,13 @@
         <v>57</v>
       </c>
       <c r="B61" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D61" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E61" s="38">
         <v>45833</v>
@@ -4209,16 +4232,16 @@
         <v>58</v>
       </c>
       <c r="B62" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D62" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E62" s="38">
-        <v>45820</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -4226,13 +4249,13 @@
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D63" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E63" s="38">
         <v>45820</v>
@@ -4243,16 +4266,16 @@
         <v>60</v>
       </c>
       <c r="B64" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D64" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E64" s="38">
-        <v>45818</v>
+        <v>45820</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -4260,16 +4283,16 @@
         <v>61</v>
       </c>
       <c r="B65" t="s">
-        <v>425</v>
-      </c>
-      <c r="C65" s="8">
-        <v>2025</v>
+        <v>424</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D65" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E65" s="38">
-        <v>45807</v>
+        <v>45818</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -4277,16 +4300,16 @@
         <v>62</v>
       </c>
       <c r="B66" t="s">
-        <v>426</v>
-      </c>
-      <c r="C66" s="8" t="s">
-        <v>4</v>
+        <v>425</v>
+      </c>
+      <c r="C66" s="8">
+        <v>2025</v>
       </c>
       <c r="D66" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="E66" s="38">
-        <v>45793</v>
+        <v>45807</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -4294,16 +4317,16 @@
         <v>63</v>
       </c>
       <c r="B67" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D67" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E67" s="38">
-        <v>45784</v>
+        <v>45793</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -4311,16 +4334,16 @@
         <v>64</v>
       </c>
       <c r="B68" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D68" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E68" s="38">
-        <v>45783</v>
+        <v>45784</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -4328,13 +4351,13 @@
         <v>65</v>
       </c>
       <c r="B69" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D69" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E69" s="38">
         <v>45783</v>
@@ -4345,16 +4368,16 @@
         <v>66</v>
       </c>
       <c r="B70" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D70" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E70" s="38">
-        <v>45771</v>
+        <v>45783</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -4362,16 +4385,16 @@
         <v>67</v>
       </c>
       <c r="B71" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D71" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E71" s="38">
-        <v>45762</v>
+        <v>45771</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -4379,16 +4402,16 @@
         <v>68</v>
       </c>
       <c r="B72" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>4</v>
       </c>
       <c r="D72" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E72" s="38">
-        <v>45750</v>
+        <v>45762</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -4396,16 +4419,16 @@
         <v>69</v>
       </c>
       <c r="B73" t="s">
-        <v>433</v>
-      </c>
-      <c r="C73" s="8">
-        <v>2025</v>
+        <v>432</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>4</v>
       </c>
       <c r="D73" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E73" s="38">
-        <v>45744</v>
+        <v>45750</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -4413,16 +4436,16 @@
         <v>70</v>
       </c>
       <c r="B74" t="s">
-        <v>110</v>
-      </c>
-      <c r="C74" s="8" t="s">
-        <v>4</v>
+        <v>433</v>
+      </c>
+      <c r="C74" s="8">
+        <v>2025</v>
       </c>
       <c r="D74" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E74" s="38">
-        <v>45743</v>
+        <v>45744</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -4430,13 +4453,13 @@
         <v>71</v>
       </c>
       <c r="B75" t="s">
-        <v>434</v>
+        <v>110</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>112</v>
+        <v>4</v>
       </c>
       <c r="D75" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E75" s="38">
         <v>45743</v>
@@ -4447,16 +4470,16 @@
         <v>72</v>
       </c>
       <c r="B76" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D76" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E76" s="38">
-        <v>45735</v>
+        <v>45743</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -4464,16 +4487,16 @@
         <v>73</v>
       </c>
       <c r="B77" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D77" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E77" s="38">
-        <v>45726</v>
+        <v>45735</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -4481,16 +4504,16 @@
         <v>74</v>
       </c>
       <c r="B78" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D78" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E78" s="38">
-        <v>45719</v>
+        <v>45726</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -4498,16 +4521,16 @@
         <v>75</v>
       </c>
       <c r="B79" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D79" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E79" s="38">
-        <v>45700</v>
+        <v>45719</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -4515,16 +4538,16 @@
         <v>76</v>
       </c>
       <c r="B80" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D80" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E80" s="38">
-        <v>45695</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -4532,16 +4555,16 @@
         <v>77</v>
       </c>
       <c r="B81" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D81" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E81" s="38">
-        <v>45694</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -4549,16 +4572,16 @@
         <v>78</v>
       </c>
       <c r="B82" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D82" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E82" s="38">
-        <v>45692</v>
+        <v>45694</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -4566,16 +4589,16 @@
         <v>79</v>
       </c>
       <c r="B83" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D83" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E83" s="38">
-        <v>45688</v>
+        <v>45692</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -4583,16 +4606,16 @@
         <v>80</v>
       </c>
       <c r="B84" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D84" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E84" s="38">
-        <v>45684</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -4600,16 +4623,16 @@
         <v>81</v>
       </c>
       <c r="B85" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D85" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E85" s="38">
-        <v>45678</v>
+        <v>45684</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -4617,16 +4640,16 @@
         <v>82</v>
       </c>
       <c r="B86" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D86" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E86" s="38">
-        <v>45672</v>
+        <v>45678</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -4634,13 +4657,13 @@
         <v>83</v>
       </c>
       <c r="B87" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D87" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E87" s="38">
         <v>45672</v>
@@ -4668,16 +4691,16 @@
         <v>85</v>
       </c>
       <c r="B89" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D89" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E89" s="38">
-        <v>45662</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -4685,16 +4708,16 @@
         <v>86</v>
       </c>
       <c r="B90" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D90" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E90" s="38">
-        <v>45660</v>
+        <v>45662</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -4702,16 +4725,16 @@
         <v>87</v>
       </c>
       <c r="B91" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D91" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E91" s="38">
-        <v>45659</v>
+        <v>45660</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -4719,16 +4742,16 @@
         <v>88</v>
       </c>
       <c r="B92" t="s">
-        <v>450</v>
-      </c>
-      <c r="C92" s="8">
-        <v>2024</v>
+        <v>449</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>114</v>
       </c>
       <c r="D92" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E92" s="38">
-        <v>45653</v>
+        <v>45659</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -4736,16 +4759,16 @@
         <v>89</v>
       </c>
       <c r="B93" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C93" s="8">
         <v>2024</v>
       </c>
       <c r="D93" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E93" s="38">
-        <v>45650</v>
+        <v>45653</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -4753,16 +4776,16 @@
         <v>90</v>
       </c>
       <c r="B94" t="s">
-        <v>452</v>
-      </c>
-      <c r="C94" s="8" t="s">
-        <v>114</v>
+        <v>451</v>
+      </c>
+      <c r="C94" s="8">
+        <v>2024</v>
       </c>
       <c r="D94" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E94" s="38">
-        <v>45643</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -4770,16 +4793,16 @@
         <v>91</v>
       </c>
       <c r="B95" t="s">
-        <v>284</v>
+        <v>452</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D95" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E95" s="38">
-        <v>45639</v>
+        <v>45643</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -4787,16 +4810,16 @@
         <v>92</v>
       </c>
       <c r="B96" t="s">
-        <v>453</v>
+        <v>284</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D96" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E96" s="38">
-        <v>45610</v>
+        <v>45639</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
@@ -4804,16 +4827,16 @@
         <v>93</v>
       </c>
       <c r="B97" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D97" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E97" s="38">
-        <v>45609</v>
+        <v>45610</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -4821,16 +4844,16 @@
         <v>94</v>
       </c>
       <c r="B98" t="s">
-        <v>455</v>
-      </c>
-      <c r="C98" s="8">
-        <v>2024</v>
+        <v>454</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>114</v>
       </c>
       <c r="D98" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E98" s="38">
-        <v>45601</v>
+        <v>45609</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
@@ -4838,16 +4861,16 @@
         <v>95</v>
       </c>
       <c r="B99" t="s">
-        <v>456</v>
-      </c>
-      <c r="C99" s="8" t="s">
-        <v>114</v>
+        <v>455</v>
+      </c>
+      <c r="C99" s="8">
+        <v>2024</v>
       </c>
       <c r="D99" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E99" s="38">
-        <v>45597</v>
+        <v>45601</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -4855,13 +4878,13 @@
         <v>96</v>
       </c>
       <c r="B100" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D100" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E100" s="38">
         <v>45597</v>
@@ -4872,16 +4895,16 @@
         <v>97</v>
       </c>
       <c r="B101" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D101" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E101" s="38">
-        <v>45593</v>
+        <v>45597</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
@@ -4889,16 +4912,16 @@
         <v>98</v>
       </c>
       <c r="B102" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D102" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E102" s="38">
-        <v>45588</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -4906,16 +4929,16 @@
         <v>99</v>
       </c>
       <c r="B103" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C103" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D103" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E103" s="38">
-        <v>45572</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -4923,16 +4946,16 @@
         <v>100</v>
       </c>
       <c r="B104" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C104" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D104" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E104" s="38">
-        <v>45562</v>
+        <v>45572</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
@@ -4940,16 +4963,16 @@
         <v>101</v>
       </c>
       <c r="B105" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D105" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E105" s="38">
-        <v>45555</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -4957,16 +4980,16 @@
         <v>102</v>
       </c>
       <c r="B106" t="s">
-        <v>463</v>
-      </c>
-      <c r="C106" s="8">
-        <v>2024</v>
+        <v>462</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>114</v>
       </c>
       <c r="D106" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E106" s="38">
-        <v>45547</v>
+        <v>45555</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
@@ -4974,16 +4997,16 @@
         <v>103</v>
       </c>
       <c r="B107" t="s">
-        <v>464</v>
-      </c>
-      <c r="C107" s="8" t="s">
-        <v>114</v>
+        <v>463</v>
+      </c>
+      <c r="C107" s="8">
+        <v>2024</v>
       </c>
       <c r="D107" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E107" s="38">
-        <v>45538</v>
+        <v>45547</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -4991,16 +5014,16 @@
         <v>104</v>
       </c>
       <c r="B108" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D108" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E108" s="38">
-        <v>45534</v>
+        <v>45538</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -5008,16 +5031,16 @@
         <v>105</v>
       </c>
       <c r="B109" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D109" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E109" s="38">
-        <v>45533</v>
+        <v>45534</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
@@ -5025,13 +5048,13 @@
         <v>106</v>
       </c>
       <c r="B110" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C110" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D110" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E110" s="38">
         <v>45533</v>
@@ -5042,16 +5065,16 @@
         <v>107</v>
       </c>
       <c r="B111" t="s">
-        <v>468</v>
-      </c>
-      <c r="C111" s="8">
-        <v>2024</v>
+        <v>467</v>
+      </c>
+      <c r="C111" s="8" t="s">
+        <v>112</v>
       </c>
       <c r="D111" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E111" s="38">
-        <v>45526</v>
+        <v>45533</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
@@ -5059,16 +5082,16 @@
         <v>108</v>
       </c>
       <c r="B112" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C112" s="8">
         <v>2024</v>
       </c>
       <c r="D112" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E112" s="38">
-        <v>45518</v>
+        <v>45526</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
@@ -5076,16 +5099,16 @@
         <v>109</v>
       </c>
       <c r="B113" t="s">
-        <v>470</v>
-      </c>
-      <c r="C113" s="8" t="s">
-        <v>114</v>
+        <v>469</v>
+      </c>
+      <c r="C113" s="8">
+        <v>2024</v>
       </c>
       <c r="D113" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E113" s="38">
-        <v>45502</v>
+        <v>45518</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
@@ -5093,16 +5116,16 @@
         <v>110</v>
       </c>
       <c r="B114" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C114" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D114" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E114" s="38">
-        <v>45498</v>
+        <v>45502</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
@@ -5110,16 +5133,16 @@
         <v>111</v>
       </c>
       <c r="B115" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C115" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D115" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E115" s="38">
-        <v>45489</v>
+        <v>45498</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -5127,16 +5150,16 @@
         <v>112</v>
       </c>
       <c r="B116" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C116" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D116" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E116" s="38">
-        <v>45469</v>
+        <v>45489</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
@@ -5144,13 +5167,13 @@
         <v>113</v>
       </c>
       <c r="B117" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C117" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D117" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E117" s="38">
         <v>45469</v>
@@ -5161,16 +5184,16 @@
         <v>114</v>
       </c>
       <c r="B118" t="s">
-        <v>202</v>
+        <v>474</v>
       </c>
       <c r="C118" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D118" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E118" s="38">
-        <v>45455</v>
+        <v>45469</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
@@ -5178,13 +5201,13 @@
         <v>115</v>
       </c>
       <c r="B119" t="s">
-        <v>475</v>
+        <v>202</v>
       </c>
       <c r="C119" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D119" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E119" s="38">
         <v>45455</v>
@@ -5195,16 +5218,16 @@
         <v>116</v>
       </c>
       <c r="B120" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C120" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D120" t="s">
-        <v>162</v>
+        <v>206</v>
       </c>
       <c r="E120" s="38">
-        <v>45449</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
@@ -5212,13 +5235,13 @@
         <v>117</v>
       </c>
       <c r="B121" t="s">
-        <v>477</v>
-      </c>
-      <c r="C121" s="8">
-        <v>2024</v>
+        <v>476</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>114</v>
       </c>
       <c r="D121" t="s">
-        <v>209</v>
+        <v>162</v>
       </c>
       <c r="E121" s="38">
         <v>45449</v>
@@ -5229,16 +5252,16 @@
         <v>118</v>
       </c>
       <c r="B122" t="s">
-        <v>478</v>
-      </c>
-      <c r="C122" s="8" t="s">
-        <v>114</v>
+        <v>477</v>
+      </c>
+      <c r="C122" s="8">
+        <v>2024</v>
       </c>
       <c r="D122" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E122" s="38">
-        <v>45446</v>
+        <v>45449</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
@@ -5246,16 +5269,16 @@
         <v>119</v>
       </c>
       <c r="B123" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C123" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D123" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E123" s="38">
-        <v>45441</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
@@ -5263,16 +5286,16 @@
         <v>120</v>
       </c>
       <c r="B124" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D124" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E124" s="38">
-        <v>45440</v>
+        <v>45441</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
@@ -5280,16 +5303,16 @@
         <v>121</v>
       </c>
       <c r="B125" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>112</v>
       </c>
       <c r="D125" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E125" s="38">
-        <v>45439</v>
+        <v>45440</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
@@ -5297,16 +5320,16 @@
         <v>122</v>
       </c>
       <c r="B126" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D126" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E126" s="38">
-        <v>45422</v>
+        <v>45439</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -5314,16 +5337,16 @@
         <v>123</v>
       </c>
       <c r="B127" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C127" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D127" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E127" s="38">
-        <v>45415</v>
+        <v>45422</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
@@ -5331,16 +5354,16 @@
         <v>124</v>
       </c>
       <c r="B128" t="s">
-        <v>285</v>
+        <v>483</v>
       </c>
       <c r="C128" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D128" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E128" s="38">
-        <v>45411</v>
+        <v>45415</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
@@ -5348,16 +5371,16 @@
         <v>125</v>
       </c>
       <c r="B129" t="s">
-        <v>484</v>
+        <v>285</v>
       </c>
       <c r="C129" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D129" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E129" s="38">
-        <v>45391</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
@@ -5365,13 +5388,13 @@
         <v>126</v>
       </c>
       <c r="B130" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C130" s="8" t="s">
         <v>114</v>
       </c>
       <c r="D130" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E130" s="38">
         <v>45391</v>
@@ -5382,16 +5405,16 @@
         <v>127</v>
       </c>
       <c r="B131" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>235</v>
+        <v>114</v>
       </c>
       <c r="D131" t="s">
-        <v>105</v>
+        <v>229</v>
       </c>
       <c r="E131" s="38">
-        <v>45379</v>
+        <v>45391</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
@@ -5399,16 +5422,16 @@
         <v>128</v>
       </c>
       <c r="B132" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D132" t="s">
-        <v>238</v>
+        <v>105</v>
       </c>
       <c r="E132" s="38">
-        <v>45378</v>
+        <v>45379</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
@@ -5416,13 +5439,13 @@
         <v>129</v>
       </c>
       <c r="B133" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D133" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E133" s="38">
         <v>45378</v>
@@ -5433,16 +5456,16 @@
         <v>130</v>
       </c>
       <c r="B134" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D134" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="E134" s="38">
-        <v>45365</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
@@ -5450,16 +5473,16 @@
         <v>131</v>
       </c>
       <c r="B135" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D135" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="E135" s="38">
-        <v>45362</v>
+        <v>45365</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
@@ -5467,13 +5490,13 @@
         <v>132</v>
       </c>
       <c r="B136" t="s">
-        <v>504</v>
+        <v>490</v>
       </c>
       <c r="C136" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D136" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E136" s="38">
         <v>45362</v>
@@ -5484,16 +5507,16 @@
         <v>133</v>
       </c>
       <c r="B137" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C137" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D137" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E137" s="38">
-        <v>45358</v>
+        <v>45362</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
@@ -5501,13 +5524,13 @@
         <v>134</v>
       </c>
       <c r="B138" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C138" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D138" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E138" s="38">
         <v>45358</v>
@@ -5518,16 +5541,16 @@
         <v>135</v>
       </c>
       <c r="B139" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C139" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D139" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E139" s="38">
-        <v>45357</v>
+        <v>45358</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
@@ -5535,16 +5558,16 @@
         <v>136</v>
       </c>
       <c r="B140" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C140" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D140" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E140" s="38">
-        <v>45350</v>
+        <v>45357</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
@@ -5552,16 +5575,16 @@
         <v>137</v>
       </c>
       <c r="B141" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C141" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D141" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E141" s="38">
-        <v>45344</v>
+        <v>45350</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
@@ -5569,16 +5592,16 @@
         <v>138</v>
       </c>
       <c r="B142" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C142" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D142" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E142" s="38">
-        <v>45336</v>
+        <v>45344</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
@@ -5586,13 +5609,13 @@
         <v>139</v>
       </c>
       <c r="B143" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C143" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D143" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E143" s="38">
         <v>45336</v>
@@ -5603,13 +5626,13 @@
         <v>140</v>
       </c>
       <c r="B144" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C144" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D144" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E144" s="38">
         <v>45336</v>
@@ -5620,16 +5643,16 @@
         <v>141</v>
       </c>
       <c r="B145" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C145" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D145" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E145" s="38">
-        <v>45334</v>
+        <v>45336</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
@@ -5637,16 +5660,16 @@
         <v>142</v>
       </c>
       <c r="B146" t="s">
-        <v>222</v>
+        <v>495</v>
       </c>
       <c r="C146" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D146" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E146" s="38">
-        <v>45331</v>
+        <v>45334</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
@@ -5654,16 +5677,16 @@
         <v>143</v>
       </c>
       <c r="B147" t="s">
-        <v>494</v>
+        <v>222</v>
       </c>
       <c r="C147" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D147" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E147" s="38">
-        <v>45324</v>
+        <v>45331</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
@@ -5671,16 +5694,16 @@
         <v>144</v>
       </c>
       <c r="B148" t="s">
-        <v>493</v>
-      </c>
-      <c r="C148" s="8">
-        <v>2024</v>
+        <v>494</v>
+      </c>
+      <c r="C148" s="8" t="s">
+        <v>236</v>
       </c>
       <c r="D148" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E148" s="38">
-        <v>45322</v>
+        <v>45324</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
@@ -5688,16 +5711,16 @@
         <v>145</v>
       </c>
       <c r="B149" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C149" s="8">
         <v>2024</v>
       </c>
       <c r="D149" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E149" s="38">
-        <v>45303</v>
+        <v>45322</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
@@ -5705,20 +5728,34 @@
         <v>146</v>
       </c>
       <c r="B150" t="s">
+        <v>492</v>
+      </c>
+      <c r="C150" s="8">
+        <v>2024</v>
+      </c>
+      <c r="D150" t="s">
+        <v>278</v>
+      </c>
+      <c r="E150" s="38">
+        <v>45303</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>147</v>
+      </c>
+      <c r="B151" t="s">
         <v>491</v>
       </c>
-      <c r="C150" s="8" t="s">
+      <c r="C151" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="D150" t="s">
+      <c r="D151" t="s">
         <v>280</v>
       </c>
-      <c r="E150" s="38">
+      <c r="E151" s="38">
         <v>45294</v>
       </c>
-    </row>
-    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B305" s="2"/>
     </row>
     <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="2"/>
@@ -5732,17 +5769,17 @@
     <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="2"/>
     </row>
-    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B312" s="2"/>
-    </row>
-    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B317" s="2"/>
-    </row>
-    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B320" s="2"/>
-    </row>
-    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B322" s="2"/>
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B310" s="2"/>
+    </row>
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B313" s="2"/>
+    </row>
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B318" s="2"/>
+    </row>
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B321" s="2"/>
     </row>
     <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="2"/>
@@ -5750,8 +5787,8 @@
     <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="2"/>
     </row>
-    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B326" s="2"/>
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B325" s="2"/>
     </row>
     <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="2"/>
@@ -5765,15 +5802,18 @@
     <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="2"/>
     </row>
-    <row r="332" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B332" s="2"/>
-    </row>
-    <row r="383" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B383" s="2"/>
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B331" s="2"/>
+    </row>
+    <row r="333" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B333" s="2"/>
+    </row>
+    <row r="384" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B384" s="2"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A25:E148">
-    <sortCondition descending="1" sortBy="icon" ref="E25:E148"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A26:E149">
+    <sortCondition descending="1" sortBy="icon" ref="E26:E149"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9623,7 +9663,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="20"/>
@@ -9672,17 +9712,17 @@
       <c r="A5" s="19">
         <v>1</v>
       </c>
-      <c r="B5" s="54" t="s">
-        <v>878</v>
-      </c>
-      <c r="C5" s="55" t="s">
+      <c r="B5" s="58" t="s">
+        <v>884</v>
+      </c>
+      <c r="C5" s="59" t="s">
         <v>819</v>
       </c>
-      <c r="D5" s="54" t="s">
-        <v>879</v>
-      </c>
-      <c r="E5" s="56">
-        <v>46164</v>
+      <c r="D5" s="58" t="s">
+        <v>885</v>
+      </c>
+      <c r="E5" s="60">
+        <v>46171</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -9690,13 +9730,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="54" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="C6" s="55" t="s">
         <v>819</v>
       </c>
       <c r="D6" s="54" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="E6" s="56">
         <v>46164</v>
@@ -9706,17 +9746,17 @@
       <c r="A7" s="19">
         <v>3</v>
       </c>
-      <c r="B7" s="34" t="s">
-        <v>876</v>
-      </c>
-      <c r="C7" s="35" t="s">
+      <c r="B7" s="54" t="s">
+        <v>880</v>
+      </c>
+      <c r="C7" s="55" t="s">
         <v>819</v>
       </c>
-      <c r="D7" s="34" t="s">
-        <v>877</v>
-      </c>
-      <c r="E7" s="49">
-        <v>46155</v>
+      <c r="D7" s="54" t="s">
+        <v>881</v>
+      </c>
+      <c r="E7" s="56">
+        <v>46164</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -9724,16 +9764,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>850</v>
+        <v>876</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>814</v>
+        <v>819</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>851</v>
-      </c>
-      <c r="E8" s="40">
-        <v>46133</v>
+        <v>877</v>
+      </c>
+      <c r="E8" s="49">
+        <v>46155</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -9741,33 +9781,33 @@
         <v>5</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="E9" s="40">
-        <v>46132</v>
+        <v>46133</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>6</v>
       </c>
-      <c r="B10" s="21" t="s">
-        <v>813</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>814</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>815</v>
-      </c>
-      <c r="E10" s="41">
-        <v>46113</v>
+      <c r="B10" s="34" t="s">
+        <v>848</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>819</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>849</v>
+      </c>
+      <c r="E10" s="40">
+        <v>46132</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -9775,92 +9815,92 @@
         <v>7</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>789</v>
+        <v>813</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>8</v>
+        <v>814</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>790</v>
+        <v>815</v>
       </c>
       <c r="E11" s="41">
-        <v>46101</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8</v>
       </c>
-      <c r="B12" s="27" t="s">
-        <v>774</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>775</v>
-      </c>
-      <c r="E12" s="45">
-        <v>46087</v>
-      </c>
-      <c r="F12" s="30"/>
-      <c r="G12" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="21" t="s">
+        <v>789</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>790</v>
+      </c>
+      <c r="E12" s="41">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="19">
         <v>9</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="C13" s="28" t="s">
         <v>4</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="E13" s="45">
         <v>46087</v>
       </c>
       <c r="F13" s="30"/>
+      <c r="G13" t="s">
+        <v>381</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>10</v>
       </c>
-      <c r="B14" t="s">
-        <v>773</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" t="s">
-        <v>772</v>
-      </c>
-      <c r="E14" s="38">
-        <v>46084</v>
-      </c>
-      <c r="F14" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="21" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="27" t="s">
+        <v>776</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>777</v>
+      </c>
+      <c r="E14" s="45">
+        <v>46087</v>
+      </c>
+      <c r="F14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19">
         <v>11</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>744</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>745</v>
-      </c>
-      <c r="E15" s="41">
-        <v>46073</v>
+      <c r="B15" t="s">
+        <v>773</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>772</v>
+      </c>
+      <c r="E15" s="38">
+        <v>46084</v>
+      </c>
+      <c r="F15" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="21" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9868,13 +9908,13 @@
         <v>12</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="E16" s="41">
         <v>46073</v>
@@ -9885,13 +9925,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="E17" s="41">
         <v>46073</v>
@@ -9902,13 +9942,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C18" s="24" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="E18" s="41">
         <v>46073</v>
@@ -9919,33 +9959,33 @@
         <v>15</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="E19" s="41">
         <v>46073</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" s="21" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>16</v>
       </c>
-      <c r="B20" t="s">
-        <v>681</v>
-      </c>
-      <c r="C20" s="8" t="s">
+      <c r="B20" s="21" t="s">
+        <v>752</v>
+      </c>
+      <c r="C20" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D20" t="s">
-        <v>385</v>
-      </c>
-      <c r="E20" s="38">
-        <v>46267</v>
+      <c r="D20" s="21" t="s">
+        <v>753</v>
+      </c>
+      <c r="E20" s="41">
+        <v>46073</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -9953,50 +9993,50 @@
         <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="E21" s="38">
-        <v>46175</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>46267</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>18</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>683</v>
+      <c r="B22" t="s">
+        <v>682</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>314</v>
-      </c>
-      <c r="E22" s="46">
-        <v>46045</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D22" t="s">
+        <v>380</v>
+      </c>
+      <c r="E22" s="38">
+        <v>46175</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="19">
         <v>19</v>
       </c>
-      <c r="B23" s="17" t="s">
-        <v>684</v>
-      </c>
-      <c r="C23" s="16" t="s">
+      <c r="B23" s="8" t="s">
+        <v>683</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="16" t="s">
-        <v>315</v>
-      </c>
-      <c r="E23" s="47">
-        <v>46024</v>
+      <c r="D23" s="8" t="s">
+        <v>314</v>
+      </c>
+      <c r="E23" s="46">
+        <v>46045</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10004,19 +10044,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E24" s="47">
         <v>46024</v>
-      </c>
-      <c r="H24" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10024,16 +10061,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E25" s="47">
-        <v>46022</v>
+        <v>46024</v>
+      </c>
+      <c r="H25" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10041,16 +10081,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E26" s="47">
-        <v>45986</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10058,16 +10098,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D27" s="17" t="s">
-        <v>319</v>
+      <c r="D27" s="16" t="s">
+        <v>318</v>
       </c>
       <c r="E27" s="47">
-        <v>45961</v>
+        <v>45986</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10075,16 +10115,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E28" s="47">
-        <v>45959</v>
+        <v>45961</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10092,13 +10132,13 @@
         <v>25</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D29" s="16" t="s">
-        <v>321</v>
+      <c r="D29" s="17" t="s">
+        <v>320</v>
       </c>
       <c r="E29" s="47">
         <v>45959</v>
@@ -10109,16 +10149,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E30" s="47">
-        <v>45957</v>
+        <v>45959</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10126,16 +10166,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D31" s="17" t="s">
-        <v>323</v>
+      <c r="D31" s="16" t="s">
+        <v>322</v>
       </c>
       <c r="E31" s="47">
-        <v>45930</v>
+        <v>45957</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10143,16 +10183,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="16" t="s">
-        <v>324</v>
+      <c r="D32" s="17" t="s">
+        <v>323</v>
       </c>
       <c r="E32" s="47">
-        <v>45924</v>
+        <v>45930</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10160,16 +10200,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>743</v>
-      </c>
-      <c r="C33" s="16">
-        <v>2025</v>
+        <v>693</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E33" s="47">
-        <v>45896</v>
+        <v>45924</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10177,16 +10217,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>742</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>4</v>
+        <v>743</v>
+      </c>
+      <c r="C34" s="16">
+        <v>2025</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E34" s="47">
-        <v>45866</v>
+        <v>45896</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10194,16 +10234,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E35" s="47">
-        <v>45860</v>
+        <v>45866</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10211,16 +10251,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E36" s="47">
-        <v>45852</v>
+        <v>45860</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10228,16 +10268,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>739</v>
-      </c>
-      <c r="C37" s="16">
-        <v>2025</v>
-      </c>
-      <c r="D37" s="17" t="s">
-        <v>329</v>
+        <v>740</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>328</v>
       </c>
       <c r="E37" s="47">
-        <v>45840</v>
+        <v>45852</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10245,16 +10285,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>738</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="D38" s="16" t="s">
-        <v>330</v>
+        <v>739</v>
+      </c>
+      <c r="C38" s="16">
+        <v>2025</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>329</v>
       </c>
       <c r="E38" s="47">
-        <v>45826</v>
+        <v>45840</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10262,16 +10302,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E39" s="47">
-        <v>45821</v>
+        <v>45826</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10279,16 +10319,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C40" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E40" s="47">
-        <v>45776</v>
+        <v>45821</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10296,16 +10336,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>735</v>
-      </c>
-      <c r="C41" s="16">
-        <v>2025</v>
+        <v>736</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>4</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E41" s="47">
-        <v>45770</v>
+        <v>45776</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10313,16 +10353,16 @@
         <v>38</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>734</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>4</v>
+        <v>735</v>
+      </c>
+      <c r="C42" s="16">
+        <v>2025</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E42" s="47">
-        <v>45768</v>
+        <v>45770</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10330,16 +10370,16 @@
         <v>39</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E43" s="47">
-        <v>45758</v>
+        <v>45768</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10347,16 +10387,16 @@
         <v>40</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="D44" s="17" t="s">
-        <v>336</v>
+        <v>4</v>
+      </c>
+      <c r="D44" s="16" t="s">
+        <v>335</v>
       </c>
       <c r="E44" s="47">
-        <v>45741</v>
+        <v>45758</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10364,16 +10404,16 @@
         <v>41</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C45" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="D45" s="16" t="s">
-        <v>337</v>
+      <c r="D45" s="17" t="s">
+        <v>336</v>
       </c>
       <c r="E45" s="47">
-        <v>45736</v>
+        <v>45741</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10381,16 +10421,16 @@
         <v>42</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E46" s="47">
-        <v>45728</v>
+        <v>45736</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10398,16 +10438,16 @@
         <v>43</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C47" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E47" s="47">
-        <v>45716</v>
+        <v>45728</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10415,16 +10455,16 @@
         <v>44</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E48" s="47">
-        <v>45701</v>
+        <v>45716</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10432,16 +10472,16 @@
         <v>45</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E49" s="47">
-        <v>45700</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10449,16 +10489,16 @@
         <v>46</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E50" s="47">
-        <v>45699</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10466,13 +10506,13 @@
         <v>47</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E51" s="47">
         <v>45699</v>
@@ -10483,16 +10523,16 @@
         <v>48</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E52" s="47">
-        <v>45686</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10500,16 +10540,16 @@
         <v>49</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C53" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E53" s="47">
-        <v>45656</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10517,13 +10557,13 @@
         <v>50</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>722</v>
-      </c>
-      <c r="C54" s="16">
-        <v>2024</v>
-      </c>
-      <c r="D54" s="17" t="s">
-        <v>346</v>
+        <v>723</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="D54" s="16" t="s">
+        <v>345</v>
       </c>
       <c r="E54" s="47">
         <v>45656</v>
@@ -10534,16 +10574,16 @@
         <v>51</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>721</v>
-      </c>
-      <c r="C55" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="D55" s="16" t="s">
-        <v>347</v>
+        <v>722</v>
+      </c>
+      <c r="C55" s="16">
+        <v>2024</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>346</v>
       </c>
       <c r="E55" s="47">
-        <v>45646</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10551,16 +10591,16 @@
         <v>52</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C56" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E56" s="47">
-        <v>45632</v>
+        <v>45646</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10568,16 +10608,16 @@
         <v>53</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C57" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E57" s="47">
-        <v>45610</v>
+        <v>45632</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10585,16 +10625,16 @@
         <v>54</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="C58" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E58" s="47">
-        <v>45582</v>
+        <v>45610</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10602,16 +10642,16 @@
         <v>55</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C59" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E59" s="47">
-        <v>45572</v>
+        <v>45582</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10619,16 +10659,16 @@
         <v>56</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D60" s="16" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E60" s="47">
-        <v>45569</v>
+        <v>45572</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10636,16 +10676,16 @@
         <v>57</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C61" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D61" s="16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E61" s="47">
-        <v>45565</v>
+        <v>45569</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10653,16 +10693,16 @@
         <v>58</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D62" s="16" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E62" s="47">
-        <v>45552</v>
+        <v>45565</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10670,16 +10710,16 @@
         <v>59</v>
       </c>
       <c r="B63" s="17" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C63" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D63" s="16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E63" s="47">
-        <v>45535</v>
+        <v>45552</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10687,16 +10727,16 @@
         <v>60</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C64" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D64" s="16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E64" s="47">
-        <v>45533</v>
+        <v>45535</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10704,16 +10744,16 @@
         <v>61</v>
       </c>
       <c r="B65" s="17" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C65" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D65" s="16" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E65" s="47">
-        <v>45526</v>
+        <v>45533</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10721,16 +10761,16 @@
         <v>62</v>
       </c>
       <c r="B66" s="17" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D66" s="16" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E66" s="47">
-        <v>45520</v>
+        <v>45526</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10738,16 +10778,16 @@
         <v>63</v>
       </c>
       <c r="B67" s="17" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C67" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E67" s="47">
-        <v>45518</v>
+        <v>45520</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10755,16 +10795,16 @@
         <v>64</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C68" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D68" s="16" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E68" s="47">
-        <v>45506</v>
+        <v>45518</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10772,16 +10812,16 @@
         <v>65</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C69" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D69" s="16" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E69" s="47">
-        <v>45498</v>
+        <v>45506</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10789,16 +10829,16 @@
         <v>66</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C70" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D70" s="16" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E70" s="47">
-        <v>45496</v>
+        <v>45498</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10806,16 +10846,16 @@
         <v>67</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C71" s="16" t="s">
         <v>114</v>
       </c>
       <c r="D71" s="16" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E71" s="47">
-        <v>45483</v>
+        <v>45496</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10823,16 +10863,16 @@
         <v>68</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C72" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D72" s="16" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E72" s="47">
-        <v>45471</v>
+        <v>45483</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10840,16 +10880,16 @@
         <v>69</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C73" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D73" s="16" t="s">
-        <v>187</v>
+        <v>364</v>
       </c>
       <c r="E73" s="47">
-        <v>45461</v>
+        <v>45471</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10857,33 +10897,33 @@
         <v>70</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>365</v>
+        <v>187</v>
       </c>
       <c r="E74" s="47">
-        <v>45455</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="19">
         <v>71</v>
       </c>
-      <c r="B75" s="23" t="s">
-        <v>701</v>
+      <c r="B75" s="17" t="s">
+        <v>702</v>
       </c>
       <c r="C75" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D75" s="16" t="s">
-        <v>214</v>
+        <v>365</v>
       </c>
       <c r="E75" s="47">
-        <v>45440</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10891,33 +10931,33 @@
         <v>72</v>
       </c>
       <c r="B76" s="23" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="C76" s="16" t="s">
         <v>112</v>
       </c>
       <c r="D76" s="16" t="s">
-        <v>366</v>
+        <v>214</v>
       </c>
       <c r="E76" s="47">
-        <v>45422</v>
+        <v>45440</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="19">
         <v>73</v>
       </c>
-      <c r="B77" s="17" t="s">
-        <v>699</v>
+      <c r="B77" s="23" t="s">
+        <v>700</v>
       </c>
       <c r="C77" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D77" s="16" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E77" s="47">
-        <v>45400</v>
+        <v>45422</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10925,16 +10965,16 @@
         <v>74</v>
       </c>
       <c r="B78" s="17" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D78" s="16" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E78" s="47">
-        <v>45384</v>
+        <v>45400</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10942,16 +10982,16 @@
         <v>75</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>235</v>
+        <v>112</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E79" s="47">
-        <v>45371</v>
+        <v>45384</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10959,16 +10999,16 @@
         <v>76</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C80" s="16" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D80" s="16" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E80" s="47">
-        <v>45369</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10976,32 +11016,49 @@
         <v>77</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C81" s="16" t="s">
         <v>236</v>
       </c>
       <c r="D81" s="16" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E81" s="47">
-        <v>45338</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <v>45369</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="19">
         <v>78</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C82" s="16" t="s">
         <v>236</v>
       </c>
       <c r="D82" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="E82" s="47">
+        <v>45338</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="19">
+        <v>79</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>694</v>
+      </c>
+      <c r="C83" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="E82" s="47">
+      <c r="E83" s="47">
         <v>45335</v>
       </c>
     </row>

</xml_diff>